<commit_message>
Swap Infosys for Sun Pharma; residual-income valuation; Phase 3 text tooling
- Universe is now HUL + Sun Pharma + ICICI Bank (group decision): pharma adds
  a defensive, non-cyclical driver and keeps a rupee hedge; lowest correlation
  with the other picks. Rationale and rejected candidates (incl. Infosys and
  Media, with certainty-equivalent figures) in docs/macro_industry.md
- Workbook rebuilt: DDM for high-payout HUL; two-stage residual income for
  low-payout Sun Pharma and for ICICI; pharma peer comps
- Pipeline refuses to publish a valuation whose stocks don't match config
- Phase 3 groundwork: document manifest and downloader, Google News RSS
  ingestion, transcript parsing (two layouts, role inference, majority vote
  across quarters), FinBERT scoring with caching; parser tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/valuation.xlsx
+++ b/workbook/valuation.xlsx
@@ -10,7 +10,7 @@
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="Inputs" sheetId="2" r:id="rId2"/>
     <sheet name="DDM" sheetId="3" r:id="rId3"/>
-    <sheet name="Bank" sheetId="4" r:id="rId4"/>
+    <sheet name="ResidualIncome" sheetId="4" r:id="rId4"/>
     <sheet name="Comps" sheetId="5" r:id="rId5"/>
     <sheet name="Sensitivity" sheetId="6" r:id="rId6"/>
     <sheet name="Summary" sheetId="7" r:id="rId7"/>
@@ -33,9 +33,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="183">
-  <si>
-    <t>Valuation workbook: Hindustan Unilever, Infosys, ICICI Bank</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="183">
+  <si>
+    <t>Valuation workbook: Hindustan Unilever, Sun Pharma, ICICI Bank</t>
   </si>
   <si>
     <t/>
@@ -62,10 +62,10 @@
     <t>Inputs: market rates, company data and model assumptions. The only sheet you need to edit.</t>
   </si>
   <si>
-    <t>DDM: two-stage dividend discount model for HUL and Infosys (BKM Ch 18).</t>
-  </si>
-  <si>
-    <t>Bank: two-stage P/B (residual income) model for ICICI Bank; terminal value = book x justified P/B.</t>
+    <t>DDM: two-stage dividend discount model for HUL, which pays out most of its earnings (BKM Ch 18).</t>
+  </si>
+  <si>
+    <t>ResidualIncome: two-stage residual-income model for Sun Pharma (low payout) and ICICI Bank (a bank); terminal value = book x justified P/B.</t>
   </si>
   <si>
     <t>Comps: peer multiples. Banks use P/B scaled by ROE because justified P/B rises with ROE.</t>
@@ -77,6 +77,12 @@
     <t>Summary: one row per stock. The Python pipeline reads this sheet; keep its layout.</t>
   </si>
   <si>
+    <t>Why different models</t>
+  </si>
+  <si>
+    <t>A DDM values only the dividends paid. For a company that reinvests two-thirds of its earnings (Sun Pharma), it misses most of the value; residual income values the book equity the company keeps building instead. Both models agree when payout is high.</t>
+  </si>
+  <si>
     <t>How to update</t>
   </si>
   <si>
@@ -137,7 +143,7 @@
     <t>Price date</t>
   </si>
   <si>
-    <t>2026-10-01</t>
+    <t>2026-10-13</t>
   </si>
   <si>
     <t>NSE close via Yahoo Finance (pipeline data/latest)</t>
@@ -149,7 +155,7 @@
     <t>Hindustan Unilever</t>
   </si>
   <si>
-    <t>Infosys</t>
+    <t>Sun Pharma</t>
   </si>
   <si>
     <t>ICICI Bank</t>
@@ -164,7 +170,7 @@
     <t>HINDUNILVR.NS</t>
   </si>
   <si>
-    <t>INFY.NS</t>
+    <t>SUNPHARMA.NS</t>
   </si>
   <si>
     <t>ICICIBANK.NS</t>
@@ -179,10 +185,13 @@
     <t>Two-stage DDM</t>
   </si>
   <si>
-    <t>Two-stage P/B (residual income)</t>
-  </si>
-  <si>
-    <t>Banks: free cash flow is not meaningful, so value book value x justified P/B</t>
+    <t>Two-stage residual income</t>
+  </si>
+  <si>
+    <t>Two-stage residual income (bank)</t>
+  </si>
+  <si>
+    <t>DDM needs a high payout (HUL). Low payout (Sun) or a bank (ICICI) -&gt; residual income</t>
   </si>
   <si>
     <t>Price (Rs)</t>
@@ -206,7 +215,7 @@
     <t>Screener P/E (TTM, excl. exceptional items)</t>
   </si>
   <si>
-    <t>Screener.in public page, read 2 Oct 2026 (consolidated)</t>
+    <t>Screener.in public page (consolidated); HUL and ICICI read 2 Oct, Sun 13 Oct 2026</t>
   </si>
   <si>
     <t>EPS, TTM (Rs) = price / Screener P/E</t>
@@ -218,19 +227,19 @@
     <t>EPS FY21 (Rs)</t>
   </si>
   <si>
-    <t>Screener.in public page, read 2 Oct 2026 (consolidated), P&amp;L table</t>
+    <t>Screener.in public page (consolidated), P&amp;L table. Sun's FY21 EPS was depressed by a Rs 3,449 Cr exceptional charge, so its 5-yr CAGR overstates growth (3-yr profit CAGR: 13%)</t>
   </si>
   <si>
     <t>EPS growth, ~5-yr CAGR</t>
   </si>
   <si>
-    <t>FY21 to TTM; a reference point for g1, not used directly</t>
+    <t>FY21 to TTM; a reference point for growth assumptions, not used directly</t>
   </si>
   <si>
     <t>Dividend per share FY26 = D0 (Rs)</t>
   </si>
   <si>
-    <t>Yahoo Finance dividends: HUL 19 (Nov-25) + 22 (Jun-26); INFY 23 (Oct-25) + 25 (Jun-26); ICICI 12 (Aug-26)</t>
+    <t>Yahoo Finance dividends: HUL 19 (Nov-25) + 22 (Jun-26); Sun 11 (Feb-26) + 5 (Jul-26); ICICI 12 (Aug-26)</t>
   </si>
   <si>
     <t>Payout ratio (DPS / EPS TTM)</t>
@@ -239,10 +248,13 @@
     <t>Book value per share (Rs)</t>
   </si>
   <si>
+    <t>Screener.in public page (consolidated)</t>
+  </si>
+  <si>
     <t>ROE, latest FY</t>
   </si>
   <si>
-    <t>Screener.in public page, read 2 Oct 2026 (consolidated) (HUL's figure includes the FY26 one-off gain)</t>
+    <t>Screener.in public page (consolidated) (HUL's figure includes the FY26 one-off gain)</t>
   </si>
   <si>
     <t>Model assumptions (review these)</t>
@@ -260,25 +272,25 @@
     <t>n/a</t>
   </si>
   <si>
-    <t>Assumption. HUL: ~5-yr sales CAGR 6.5-7% with flat margins. INFY: between 5-yr EPS CAGR (~10%) and 3-yr profit growth (8%)</t>
-  </si>
-  <si>
-    <t>ROE in high-growth phase (bank)</t>
-  </si>
-  <si>
-    <t>Assumption: FY26 ROE held for N years (3-yr average was 17%)</t>
-  </si>
-  <si>
-    <t>Payout in high-growth phase (bank)</t>
-  </si>
-  <si>
-    <t>Assumption: FY26 payout per Screener (16%)</t>
-  </si>
-  <si>
-    <t>Stable ROE after year N (bank)</t>
-  </si>
-  <si>
-    <t>Assumption: ROE fades toward the peer range (11-14%) but stays above it</t>
+    <t>Assumption. HUL: ~5-yr sales CAGR 6.5-7% with flat margins</t>
+  </si>
+  <si>
+    <t>ROE in high-growth phase (residual income)</t>
+  </si>
+  <si>
+    <t>Assumption. Sun: 5-yr average ROE 16%. ICICI: FY26 ROE (3-yr average 17%)</t>
+  </si>
+  <si>
+    <t>Payout in high-growth phase (residual income)</t>
+  </si>
+  <si>
+    <t>Assumption: FY26 payout per Screener (Sun 33%, ICICI 16%)</t>
+  </si>
+  <si>
+    <t>Stable ROE after year N (residual income)</t>
+  </si>
+  <si>
+    <t>Assumption. Sun: 10-yr average ROE 14%. ICICI: fades toward peers (11-14%) but stays above</t>
   </si>
   <si>
     <t>Terminal growth g2 (keep at or below rf)</t>
@@ -293,7 +305,7 @@
     <t>Check: g2 below r</t>
   </si>
   <si>
-    <t>Two-stage dividend discount model: Hindustan Unilever and Infosys</t>
+    <t>Two-stage dividend discount model: Hindustan Unilever</t>
   </si>
   <si>
     <t>Dividends grow at g1 for N years, then at g2 for ever. Value = PV of dividends in years 1-10 + PV of the terminal value at year 10. Years after N already grow at g2, so any N from 1 to 10 gives the textbook two-stage value.</t>
@@ -323,22 +335,13 @@
     <t>Year</t>
   </si>
   <si>
-    <t>HUL growth</t>
-  </si>
-  <si>
-    <t>HUL dividend (Rs)</t>
-  </si>
-  <si>
-    <t>HUL PV (Rs)</t>
-  </si>
-  <si>
-    <t>INFY growth</t>
-  </si>
-  <si>
-    <t>INFY dividend (Rs)</t>
-  </si>
-  <si>
-    <t>INFY PV (Rs)</t>
+    <t>Growth</t>
+  </si>
+  <si>
+    <t>Dividend (Rs)</t>
+  </si>
+  <si>
+    <t>PV (Rs)</t>
   </si>
   <si>
     <t>Results</t>
@@ -374,10 +377,10 @@
     <t>Reverse DDM: the constant growth g at which Gordon's formula D0(1+g)/(r-g) equals today's price, i.e. g = (r x P - D0) / (P + D0).</t>
   </si>
   <si>
-    <t>ICICI Bank: two-stage P/B (residual income) model</t>
-  </si>
-  <si>
-    <t>Book value compounds at ROE x retention. For N years the bank keeps its current ROE and payout; afterwards payout = 1 - g2/ROE, just enough retention to grow book at g2. Terminal value = book value x justified P/B, where justified P/B = (ROE - g) / (r - g).</t>
+    <t>Two-stage residual-income (P/B) model: Sun Pharma and ICICI Bank</t>
+  </si>
+  <si>
+    <t>Book value compounds at ROE x retention. For N years the company keeps its current ROE and payout; afterwards payout = 1 - g2/ROE, just enough retention to grow book at g2. Terminal value = book value x justified P/B, where justified P/B = (ROE - g) / (r - g). Implied growth solves single-stage P/B = (ROE - g)/(r - g): g = (r x P/B - ROE) / (P/B - 1).</t>
   </si>
   <si>
     <t>Book value per share now (Rs)</t>
@@ -434,13 +437,10 @@
     <t>Check: closed-form value (Rs)</t>
   </si>
   <si>
-    <t>Implied growth solves single-stage P/B = (ROE - g) / (r - g) for g: g = (r x P/B - ROE) / (P/B - 1).</t>
-  </si>
-  <si>
     <t>Peer multiples</t>
   </si>
   <si>
-    <t>Peer figures: Screener.in public page, read 2 Oct 2026 (consolidated). P/E is Screener's TTM P/E.</t>
+    <t>Peer figures: Screener.in public page (consolidated), read 2 Oct (FMCG, banks) and 13 Oct 2026 (pharma). P/E is Screener's TTM P/E.</t>
   </si>
   <si>
     <t>FMCG peers for Hindustan Unilever</t>
@@ -470,22 +470,22 @@
     <t>HUL value at median P/E (Rs)</t>
   </si>
   <si>
-    <t>IT services peers for Infosys</t>
-  </si>
-  <si>
-    <t>TCS</t>
-  </si>
-  <si>
-    <t>HCL Technologies</t>
-  </si>
-  <si>
-    <t>Wipro</t>
-  </si>
-  <si>
-    <t>Infosys EPS, TTM (Rs)</t>
-  </si>
-  <si>
-    <t>Infosys value at median P/E (Rs)</t>
+    <t>Pharma peers for Sun Pharma</t>
+  </si>
+  <si>
+    <t>Cipla</t>
+  </si>
+  <si>
+    <t>Dr Reddy's Laboratories</t>
+  </si>
+  <si>
+    <t>Divi's Laboratories</t>
+  </si>
+  <si>
+    <t>Sun Pharma EPS, TTM (Rs)</t>
+  </si>
+  <si>
+    <t>Sun Pharma value at median P/E (Rs)</t>
   </si>
   <si>
     <t>Private bank peers for ICICI Bank</t>
@@ -539,10 +539,10 @@
     <t>r  \  g2</t>
   </si>
   <si>
-    <t>Infosys (two-stage DDM)</t>
-  </si>
-  <si>
-    <t>ICICI Bank (two-stage P/B)</t>
+    <t>Sun Pharma (two-stage residual income)</t>
+  </si>
+  <si>
+    <t>ICICI Bank (two-stage residual income)</t>
   </si>
   <si>
     <t>ticker</t>
@@ -598,7 +598,7 @@
     <numFmt numFmtId="182" formatCode="&quot;₹&quot;#,##0"/>
     <numFmt numFmtId="183" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -647,6 +647,12 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -1132,31 +1138,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1165,119 +1168,122 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1302,8 +1308,9 @@
     <xf numFmtId="183" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="183" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="181" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1653,7 +1660,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
@@ -1751,16 +1758,16 @@
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
-      <c r="A20" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
     <row r="21" spans="1:1">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="7" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1771,27 +1778,42 @@
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="10" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1">
-      <c r="A24" s="7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="7" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="7" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1806,431 +1828,431 @@
   <dimension ref="A1:E33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="95" customWidth="1"/>
+    <col min="5" max="5" width="100" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.6" spans="1:5">
       <c r="A1" s="8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="18">
         <v>0.055199</v>
       </c>
-      <c r="E5" s="23" t="s">
-        <v>28</v>
+      <c r="E5" s="24" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="18">
         <v>0.0708</v>
       </c>
-      <c r="E6" s="23" t="s">
-        <v>30</v>
+      <c r="E6" s="24" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="24">
+        <v>33</v>
+      </c>
+      <c r="B7" s="25">
         <v>0.15</v>
       </c>
-      <c r="E7" s="23" t="s">
-        <v>32</v>
+      <c r="E7" s="24" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" s="23" t="s">
         <v>35</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="B11" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="C11" s="26" t="s">
         <v>45</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="B12" s="26" t="s">
         <v>49</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B13" s="15">
-        <v>1836</v>
+        <v>1861.9</v>
       </c>
       <c r="C13" s="15">
-        <v>1035</v>
+        <v>1759.8</v>
       </c>
       <c r="D13" s="15">
-        <v>1310.6</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>51</v>
+        <v>1350.5</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B14" s="14">
-        <v>0.6004</v>
+        <v>0.6016</v>
       </c>
       <c r="C14" s="14">
-        <v>0.8211</v>
+        <v>0.6454</v>
       </c>
       <c r="D14" s="14">
-        <v>1.2949</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>53</v>
+        <v>1.2928</v>
+      </c>
+      <c r="E14" s="24" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B15" s="5">
         <f>$B$5+B14*$B$6</f>
-        <v>0.09770732</v>
+        <v>0.09779228</v>
       </c>
       <c r="C15" s="5">
         <f>$B$5+C14*$B$6</f>
-        <v>0.11333288</v>
+        <v>0.10089332</v>
       </c>
       <c r="D15" s="5">
         <f>$B$5+D14*$B$6</f>
-        <v>0.14687792</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>55</v>
+        <v>0.14672924</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B16" s="14">
         <v>39.1</v>
       </c>
       <c r="C16" s="14">
-        <v>13.5</v>
+        <v>33.4</v>
       </c>
       <c r="D16" s="14">
         <v>16.8</v>
       </c>
-      <c r="E16" s="23" t="s">
-        <v>57</v>
+      <c r="E16" s="24" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B17" s="6">
         <f>B13/B16</f>
-        <v>46.9565217391304</v>
+        <v>47.618925831202</v>
       </c>
       <c r="C17" s="6">
         <f>C13/C16</f>
-        <v>76.6666666666667</v>
+        <v>52.688622754491</v>
       </c>
       <c r="D17" s="6">
         <f>D13/D16</f>
-        <v>78.0119047619048</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>59</v>
+        <v>80.3869047619048</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B18" s="15">
         <v>34.03</v>
       </c>
       <c r="C18" s="15">
-        <v>45.42</v>
+        <v>12.1</v>
       </c>
       <c r="D18" s="15">
         <v>26.58</v>
       </c>
-      <c r="E18" s="23" t="s">
-        <v>61</v>
+      <c r="E18" s="24" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B19" s="5">
         <f>(B17/B18)^(1/5)-1</f>
-        <v>0.0665145729752543</v>
+        <v>0.0695067480307374</v>
       </c>
       <c r="C19" s="5">
         <f>(C17/C18)^(1/5)-1</f>
-        <v>0.110380663601837</v>
+        <v>0.342104384786903</v>
       </c>
       <c r="D19" s="5">
         <f>(D17/D18)^(1/5)-1</f>
-        <v>0.240284113772609</v>
-      </c>
-      <c r="E19" s="23" t="s">
-        <v>63</v>
+        <v>0.247745654518664</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B20" s="15">
         <v>41</v>
       </c>
       <c r="C20" s="15">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="D20" s="15">
         <v>12</v>
       </c>
-      <c r="E20" s="23" t="s">
-        <v>65</v>
+      <c r="E20" s="24" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B21" s="5">
         <f>B20/B17</f>
-        <v>0.873148148148148</v>
+        <v>0.861002202051668</v>
       </c>
       <c r="C21" s="5">
         <f>C20/C17</f>
-        <v>0.626086956521739</v>
+        <v>0.303670871689965</v>
       </c>
       <c r="D21" s="5">
         <f>D20/D17</f>
-        <v>0.153822676636655</v>
-      </c>
-      <c r="E21" s="23" t="s">
+        <v>0.149278045168456</v>
+      </c>
+      <c r="E21" s="24" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B22" s="15">
         <v>207</v>
       </c>
       <c r="C22" s="15">
-        <v>225</v>
+        <v>348</v>
       </c>
       <c r="D22" s="15">
         <v>527</v>
       </c>
-      <c r="E22" s="23" t="s">
-        <v>57</v>
+      <c r="E22" s="24" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B23" s="18">
         <v>0.31</v>
       </c>
       <c r="C23" s="18">
-        <v>0.319</v>
+        <v>0.16</v>
       </c>
       <c r="D23" s="18">
         <v>0.159</v>
       </c>
-      <c r="E23" s="23" t="s">
-        <v>69</v>
+      <c r="E23" s="24" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B26" s="26">
+        <v>75</v>
+      </c>
+      <c r="B26" s="27">
         <v>5</v>
       </c>
-      <c r="C26" s="26">
+      <c r="C26" s="27">
         <v>5</v>
       </c>
-      <c r="D26" s="26">
+      <c r="D26" s="27">
         <v>5</v>
       </c>
-      <c r="E26" s="23" t="s">
-        <v>72</v>
+      <c r="E26" s="24" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B27" s="24">
+        <v>77</v>
+      </c>
+      <c r="B27" s="25">
         <v>0.07</v>
       </c>
-      <c r="C27" s="24">
-        <v>0.08</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" s="23" t="s">
-        <v>75</v>
+      <c r="C27" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B28" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D28" s="24">
+        <v>80</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="25">
         <v>0.16</v>
       </c>
-      <c r="E28" s="23" t="s">
-        <v>77</v>
+      <c r="D28" s="25">
+        <v>0.16</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C29" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D29" s="24">
+      <c r="C29" s="25">
+        <v>0.33</v>
+      </c>
+      <c r="D29" s="25">
         <v>0.16</v>
       </c>
-      <c r="E29" s="23" t="s">
-        <v>79</v>
+      <c r="E29" s="24" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B30" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="D30" s="24">
+        <v>84</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="25">
+        <v>0.14</v>
+      </c>
+      <c r="D30" s="25">
         <v>0.15</v>
       </c>
-      <c r="E30" s="23" t="s">
-        <v>81</v>
+      <c r="E30" s="24" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="B31" s="24">
+        <v>86</v>
+      </c>
+      <c r="B31" s="25">
         <v>0.055</v>
       </c>
-      <c r="C31" s="24">
+      <c r="C31" s="25">
         <v>0.055</v>
       </c>
-      <c r="D31" s="24">
+      <c r="D31" s="25">
         <v>0.055</v>
       </c>
-      <c r="E31" s="23" t="s">
-        <v>83</v>
+      <c r="E31" s="24" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B32" s="7" t="str">
         <f>IF(B31&lt;=$B$5,"OK","g2 above rf")</f>
@@ -2244,13 +2266,13 @@
         <f>IF(D31&lt;=$B$5,"OK","g2 above rf")</f>
         <v>OK</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="E32" s="24" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="7" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B33" s="7" t="str">
         <f>IF(B31&lt;B15,"OK","g2 must be below r")</f>
@@ -2264,7 +2286,7 @@
         <f>IF(D31&lt;D15,"OK","g2 must be below r")</f>
         <v>OK</v>
       </c>
-      <c r="E33" s="23" t="s">
+      <c r="E33" s="24" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2277,140 +2299,102 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G36"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="6"/>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
-    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.6" spans="1:7">
+    <row r="1" ht="17.6" spans="1:4">
       <c r="A1" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="7" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B5" s="3">
         <f>Inputs!B20</f>
         <v>41</v>
       </c>
-      <c r="C5" s="3">
-        <f>Inputs!C20</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="7" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B6" s="4">
         <f>Inputs!B15</f>
-        <v>0.09770732</v>
-      </c>
-      <c r="C6" s="4">
-        <f>Inputs!C15</f>
-        <v>0.11333288</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>0.09779228</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B7" s="4">
         <f>Inputs!B27</f>
         <v>0.07</v>
       </c>
-      <c r="C7" s="4">
-        <f>Inputs!C27</f>
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="22">
+        <v>96</v>
+      </c>
+      <c r="B8" s="23">
         <f>Inputs!B26</f>
         <v>5</v>
       </c>
-      <c r="C8" s="22">
-        <f>Inputs!C26</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="7" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B9" s="4">
         <f>Inputs!B31</f>
         <v>0.055</v>
       </c>
-      <c r="C9" s="4">
-        <f>Inputs!C31</f>
-        <v>0.055</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3">
         <f>Inputs!B13</f>
-        <v>1836</v>
-      </c>
-      <c r="C10" s="3">
-        <f>Inputs!C13</f>
-        <v>1035</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>1861.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="7">
         <v>0</v>
       </c>
@@ -2418,12 +2402,8 @@
         <f>B5</f>
         <v>41</v>
       </c>
-      <c r="F13" s="6">
-        <f>C5</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="7">
         <v>1</v>
       </c>
@@ -2437,22 +2417,10 @@
       </c>
       <c r="D14" s="6">
         <f t="shared" ref="D14:D23" si="2">C14/(1+$B$6)^A14</f>
-        <v>39.9651156557834</v>
-      </c>
-      <c r="E14" s="5">
-        <f t="shared" ref="E14:E23" si="3">IF(A14&lt;=$C$8,$C$7,$C$9)</f>
-        <v>0.08</v>
-      </c>
-      <c r="F14" s="6">
-        <f t="shared" ref="F14:F23" si="4">F13*(1+E14)</f>
-        <v>51.84</v>
-      </c>
-      <c r="G14" s="6">
-        <f t="shared" ref="G14:G23" si="5">F14/(1+$C$6)^A14</f>
-        <v>46.562893211238</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+        <v>39.9620226879351</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="7">
         <v>2</v>
       </c>
@@ -2466,22 +2434,10 @@
       </c>
       <c r="D15" s="6">
         <f t="shared" si="2"/>
-        <v>38.9563529117107</v>
-      </c>
-      <c r="E15" s="5">
-        <f t="shared" si="3"/>
-        <v>0.08</v>
-      </c>
-      <c r="F15" s="6">
-        <f t="shared" si="4"/>
-        <v>55.9872</v>
-      </c>
-      <c r="G15" s="6">
-        <f t="shared" si="5"/>
-        <v>45.1688130041906</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>38.9503233490498</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="7">
         <v>3</v>
       </c>
@@ -2495,22 +2451,10 @@
       </c>
       <c r="D16" s="6">
         <f t="shared" si="2"/>
-        <v>37.9730524303423</v>
-      </c>
-      <c r="E16" s="5">
-        <f t="shared" si="3"/>
-        <v>0.08</v>
-      </c>
-      <c r="F16" s="6">
-        <f t="shared" si="4"/>
-        <v>60.466176</v>
-      </c>
-      <c r="G16" s="6">
-        <f t="shared" si="5"/>
-        <v>43.8164711748438</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>37.9642367165155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="7">
         <v>4</v>
       </c>
@@ -2524,22 +2468,10 @@
       </c>
       <c r="D17" s="6">
         <f t="shared" si="2"/>
-        <v>37.0145715166282</v>
-      </c>
-      <c r="E17" s="5">
-        <f t="shared" si="3"/>
-        <v>0.08</v>
-      </c>
-      <c r="F17" s="6">
-        <f t="shared" si="4"/>
-        <v>65.30347008</v>
-      </c>
-      <c r="G17" s="6">
-        <f t="shared" si="5"/>
-        <v>42.5046180876571</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+        <v>37.0031143657446</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="7">
         <v>5</v>
       </c>
@@ -2553,22 +2485,10 @@
       </c>
       <c r="D18" s="6">
         <f t="shared" si="2"/>
-        <v>36.0802836978368</v>
-      </c>
-      <c r="E18" s="5">
-        <f t="shared" si="3"/>
-        <v>0.08</v>
-      </c>
-      <c r="F18" s="6">
-        <f t="shared" si="4"/>
-        <v>70.5277476864</v>
-      </c>
-      <c r="G18" s="6">
-        <f t="shared" si="5"/>
-        <v>41.232041520834</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+        <v>36.0663242880035</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="7">
         <v>6</v>
       </c>
@@ -2582,22 +2502,10 @@
       </c>
       <c r="D19" s="6">
         <f t="shared" si="2"/>
-        <v>34.6765468423931</v>
-      </c>
-      <c r="E19" s="5">
-        <f t="shared" si="3"/>
-        <v>0.055</v>
-      </c>
-      <c r="F19" s="6">
-        <f t="shared" si="4"/>
-        <v>74.406773809152</v>
-      </c>
-      <c r="G19" s="6">
-        <f t="shared" si="5"/>
-        <v>39.0716959733371</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+        <v>34.6604478980702</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="7">
         <v>7</v>
       </c>
@@ -2611,22 +2519,10 @@
       </c>
       <c r="D20" s="6">
         <f t="shared" si="2"/>
-        <v>33.3274236694757</v>
-      </c>
-      <c r="E20" s="5">
-        <f t="shared" si="3"/>
-        <v>0.055</v>
-      </c>
-      <c r="F20" s="6">
-        <f t="shared" si="4"/>
-        <v>78.4991463686554</v>
-      </c>
-      <c r="G20" s="6">
-        <f t="shared" si="5"/>
-        <v>37.0245413499965</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+        <v>33.3093730012968</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="7">
         <v>8</v>
       </c>
@@ -2640,22 +2536,10 @@
       </c>
       <c r="D21" s="6">
         <f t="shared" si="2"/>
-        <v>32.0307893831817</v>
-      </c>
-      <c r="E21" s="5">
-        <f t="shared" si="3"/>
-        <v>0.055</v>
-      </c>
-      <c r="F21" s="6">
-        <f t="shared" si="4"/>
-        <v>82.8165994189314</v>
-      </c>
-      <c r="G21" s="6">
-        <f t="shared" si="5"/>
-        <v>35.0846470322931</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+        <v>32.0109634186607</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="7">
         <v>9</v>
       </c>
@@ -2669,22 +2553,10 @@
       </c>
       <c r="D22" s="6">
         <f t="shared" si="2"/>
-        <v>30.784601854761</v>
-      </c>
-      <c r="E22" s="5">
-        <f t="shared" si="3"/>
-        <v>0.055</v>
-      </c>
-      <c r="F22" s="6">
-        <f t="shared" si="4"/>
-        <v>87.3715123869726</v>
-      </c>
-      <c r="G22" s="6">
-        <f t="shared" si="5"/>
-        <v>33.2463931354198</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+        <v>30.7631662400532</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" s="7">
         <v>10</v>
       </c>
@@ -2698,165 +2570,110 @@
       </c>
       <c r="D23" s="6">
         <f t="shared" si="2"/>
-        <v>29.5868984063738</v>
-      </c>
-      <c r="E23" s="5">
-        <f t="shared" si="3"/>
-        <v>0.055</v>
-      </c>
-      <c r="F23" s="6">
-        <f t="shared" si="4"/>
-        <v>92.1769455682561</v>
-      </c>
-      <c r="G23" s="6">
-        <f t="shared" si="5"/>
-        <v>31.5044542274436</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+        <v>29.5640085784318</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B26" s="6">
         <f>SUM(D14:D23)</f>
-        <v>350.395636368487</v>
-      </c>
-      <c r="C26" s="6">
-        <f>SUM(G14:G23)</f>
-        <v>395.216568717253</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
+        <v>350.253980543761</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B27" s="6">
         <f>C23*(1+B9)/(B6-B9)</f>
-        <v>1856.58648129811</v>
-      </c>
-      <c r="C27" s="6">
-        <f>F23*(1+C9)/(C6-C9)</f>
-        <v>1667.09885701701</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+        <v>1852.90040550474</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B28" s="6">
         <f>B27/(1+B6)^10</f>
-        <v>730.885895409133</v>
-      </c>
-      <c r="C28" s="6">
-        <f>C27/(1+C6)^10</f>
-        <v>569.784985928227</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+        <v>728.870465659822</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B29" s="17">
         <f>B26+B28</f>
-        <v>1081.28153177762</v>
-      </c>
-      <c r="C29" s="17">
-        <f>C26+C28</f>
-        <v>965.00155464548</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
+        <v>1079.12444620358</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B30" s="6">
         <f>B10</f>
-        <v>1836</v>
-      </c>
-      <c r="C30" s="6">
-        <f>C10</f>
-        <v>1035</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+        <v>1861.9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B31" s="5">
         <f>B29/B30-1</f>
-        <v>-0.411066703824826</v>
-      </c>
-      <c r="C31" s="5">
-        <f>C29/C30-1</f>
-        <v>-0.0676313481686179</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+        <v>-0.420417613081485</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B32" s="5">
         <f>B28/B29</f>
-        <v>0.675944121793666</v>
-      </c>
-      <c r="C32" s="5">
-        <f>C28/C29</f>
-        <v>0.590449811386628</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
+        <v>0.675427628596523</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
       <c r="A33" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B33" s="5">
         <f>(B6*B30-B5)/(B30+B5)</f>
-        <v>0.0737296960681939</v>
-      </c>
-      <c r="C33" s="5">
-        <f>(C6*C30-C5)/(C30+C5)</f>
-        <v>0.0639884864265928</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
+        <v>0.074139180268012</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
       <c r="A34" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B34" s="6">
         <f>B5*(1+B7)/(B6-B7)*(1-((1+B7)/(1+B6))^B8)+B5*(1+B7)^B8*(1+B9)/((B6-B9)*(1+B6)^B8)</f>
-        <v>1081.28153177762</v>
-      </c>
-      <c r="C34" s="6">
-        <f>C5*(1+C7)/(C6-C7)*(1-((1+C7)/(1+C6))^C8)+C5*(1+C7)^C8*(1+C9)/((C6-C9)*(1+C6)^C8)</f>
-        <v>965.00155464548</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+        <v>1079.12444620358</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
       <c r="A35" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B35" s="20">
         <f>ROUND(B29-B34,6)</f>
         <v>0</v>
       </c>
-      <c r="C35" s="20">
-        <f>ROUND(C29-C34,6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
+    </row>
+    <row r="36" spans="1:2">
       <c r="A36" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2868,7 +2685,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -2883,202 +2700,175 @@
   <sheetData>
     <row r="1" ht="17.6" spans="1:8">
       <c r="A1" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>39</v>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" ht="15" spans="1:8">
+      <c r="A4" s="22" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B5" s="3">
-        <f>Inputs!D22</f>
-        <v>527</v>
+        <f>Inputs!C22</f>
+        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="7" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B6" s="4">
-        <f>Inputs!D15</f>
-        <v>0.14687792</v>
+        <f>Inputs!C15</f>
+        <v>0.10089332</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="22">
-        <f>Inputs!D26</f>
+        <v>96</v>
+      </c>
+      <c r="B7" s="23">
+        <f>Inputs!C26</f>
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B8" s="4">
-        <f>Inputs!D28</f>
+        <f>Inputs!C28</f>
         <v>0.16</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B9" s="4">
-        <f>Inputs!D29</f>
-        <v>0.16</v>
+        <f>Inputs!C29</f>
+        <v>0.33</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B10" s="4">
-        <f>Inputs!D30</f>
-        <v>0.15</v>
+        <f>Inputs!C30</f>
+        <v>0.14</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="7" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B11" s="4">
-        <f>Inputs!D31</f>
+        <f>Inputs!C31</f>
         <v>0.055</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B12" s="3">
-        <f>Inputs!D13</f>
-        <v>1310.6</v>
+        <f>Inputs!C13</f>
+        <v>1759.8</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="B13" s="5">
-        <f>1-B11/B10</f>
-        <v>0.633333333333333</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B15" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="4">
+        <f>Inputs!C23</f>
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="B14" s="5">
+        <f>1-$B$11/$B$10</f>
+        <v>0.607142857142857</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="7">
-        <v>1</v>
-      </c>
-      <c r="B16" s="6">
-        <f>$B$5</f>
-        <v>527</v>
-      </c>
-      <c r="C16" s="5">
-        <f t="shared" ref="C16:C25" si="0">IF(A16&lt;=$B$7,$B$8,$B$10)</f>
-        <v>0.16</v>
-      </c>
-      <c r="D16" s="6">
-        <f t="shared" ref="D16:D25" si="1">B16*C16</f>
-        <v>84.32</v>
-      </c>
-      <c r="E16" s="5">
-        <f t="shared" ref="E16:E25" si="2">IF(A16&lt;=$B$7,$B$9,$B$13)</f>
-        <v>0.16</v>
-      </c>
-      <c r="F16" s="6">
-        <f t="shared" ref="F16:F25" si="3">D16*E16</f>
-        <v>13.4912</v>
-      </c>
-      <c r="G16" s="6">
-        <f t="shared" ref="G16:G25" si="4">B16+D16-F16</f>
-        <v>597.8288</v>
-      </c>
-      <c r="H16" s="6">
-        <f t="shared" ref="H16:H25" si="5">F16/(1+$B$6)^A16</f>
-        <v>11.7634141914599</v>
+      <c r="H16" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" s="6">
-        <f t="shared" ref="B17:B25" si="6">G16</f>
-        <v>597.8288</v>
+        <f>$B$5</f>
+        <v>348</v>
       </c>
       <c r="C17" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C17:C26" si="0">IF(A17&lt;=$B$7,$B$8,$B$10)</f>
         <v>0.16</v>
       </c>
       <c r="D17" s="6">
-        <f t="shared" si="1"/>
-        <v>95.652608</v>
+        <f t="shared" ref="D17:D26" si="1">B17*C17</f>
+        <v>55.68</v>
       </c>
       <c r="E17" s="5">
-        <f t="shared" si="2"/>
-        <v>0.16</v>
+        <f t="shared" ref="E17:E26" si="2">IF(A17&lt;=$B$7,$B$9,$B$14)</f>
+        <v>0.33</v>
       </c>
       <c r="F17" s="6">
-        <f t="shared" si="3"/>
-        <v>15.30441728</v>
+        <f t="shared" ref="F17:F26" si="3">D17*E17</f>
+        <v>18.3744</v>
       </c>
       <c r="G17" s="6">
-        <f t="shared" si="4"/>
-        <v>678.17699072</v>
+        <f t="shared" ref="G17:G26" si="4">B17+D17-F17</f>
+        <v>385.3056</v>
       </c>
       <c r="H17" s="6">
-        <f t="shared" si="5"/>
-        <v>11.6354293914666</v>
+        <f t="shared" ref="H17:H26" si="5">F17/(1+$B$6)^A17</f>
+        <v>16.6904455374477</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18" s="6">
-        <f t="shared" si="6"/>
-        <v>678.17699072</v>
+        <f t="shared" ref="B18:B26" si="6">G17</f>
+        <v>385.3056</v>
       </c>
       <c r="C18" s="5">
         <f t="shared" si="0"/>
@@ -3086,32 +2876,32 @@
       </c>
       <c r="D18" s="6">
         <f t="shared" si="1"/>
-        <v>108.5083185152</v>
+        <v>61.648896</v>
       </c>
       <c r="E18" s="5">
         <f t="shared" si="2"/>
-        <v>0.16</v>
+        <v>0.33</v>
       </c>
       <c r="F18" s="6">
         <f t="shared" si="3"/>
-        <v>17.361330962432</v>
+        <v>20.34413568</v>
       </c>
       <c r="G18" s="6">
         <f t="shared" si="4"/>
-        <v>769.323978272768</v>
+        <v>426.61036032</v>
       </c>
       <c r="H18" s="6">
         <f t="shared" si="5"/>
-        <v>11.5088370536244</v>
+        <v>16.7860599781477</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B19" s="6">
         <f t="shared" si="6"/>
-        <v>769.323978272768</v>
+        <v>426.61036032</v>
       </c>
       <c r="C19" s="5">
         <f t="shared" si="0"/>
@@ -3119,32 +2909,32 @@
       </c>
       <c r="D19" s="6">
         <f t="shared" si="1"/>
-        <v>123.091836523643</v>
+        <v>68.2576576512</v>
       </c>
       <c r="E19" s="5">
         <f t="shared" si="2"/>
-        <v>0.16</v>
+        <v>0.33</v>
       </c>
       <c r="F19" s="6">
         <f t="shared" si="3"/>
-        <v>19.6946938437829</v>
+        <v>22.525027024896</v>
       </c>
       <c r="G19" s="6">
         <f t="shared" si="4"/>
-        <v>872.721120952628</v>
+        <v>472.342990946304</v>
       </c>
       <c r="H19" s="6">
         <f t="shared" si="5"/>
-        <v>11.3836220280809</v>
+        <v>16.8822221646373</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20" s="6">
         <f t="shared" si="6"/>
-        <v>872.721120952628</v>
+        <v>472.342990946304</v>
       </c>
       <c r="C20" s="5">
         <f t="shared" si="0"/>
@@ -3152,268 +2942,292 @@
       </c>
       <c r="D20" s="6">
         <f t="shared" si="1"/>
-        <v>139.63537935242</v>
+        <v>75.5748785514086</v>
       </c>
       <c r="E20" s="5">
         <f t="shared" si="2"/>
-        <v>0.16</v>
+        <v>0.33</v>
       </c>
       <c r="F20" s="6">
         <f t="shared" si="3"/>
-        <v>22.3416606963873</v>
+        <v>24.9397099219649</v>
       </c>
       <c r="G20" s="6">
         <f t="shared" si="4"/>
-        <v>990.014839608661</v>
+        <v>522.978159575748</v>
       </c>
       <c r="H20" s="6">
         <f t="shared" si="5"/>
-        <v>11.2597693298123</v>
+        <v>16.978935234784</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B21" s="6">
         <f t="shared" si="6"/>
-        <v>990.014839608661</v>
+        <v>522.978159575748</v>
       </c>
       <c r="C21" s="5">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="D21" s="6">
         <f t="shared" si="1"/>
-        <v>148.502225941299</v>
+        <v>83.6765055321196</v>
       </c>
       <c r="E21" s="5">
         <f t="shared" si="2"/>
-        <v>0.633333333333333</v>
+        <v>0.33</v>
       </c>
       <c r="F21" s="6">
         <f t="shared" si="3"/>
-        <v>94.0514097628228</v>
+        <v>27.6132468255995</v>
       </c>
       <c r="G21" s="6">
         <f t="shared" si="4"/>
-        <v>1044.46565578714</v>
+        <v>579.041418282268</v>
       </c>
       <c r="H21" s="6">
         <f t="shared" si="5"/>
-        <v>41.3296911327705</v>
+        <v>17.0762023444314</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B22" s="6">
         <f t="shared" si="6"/>
-        <v>1044.46565578714</v>
+        <v>579.041418282268</v>
       </c>
       <c r="C22" s="5">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="D22" s="6">
         <f t="shared" si="1"/>
-        <v>156.669848368071</v>
+        <v>81.0657985595175</v>
       </c>
       <c r="E22" s="5">
         <f t="shared" si="2"/>
-        <v>0.633333333333333</v>
+        <v>0.607142857142857</v>
       </c>
       <c r="F22" s="6">
         <f t="shared" si="3"/>
-        <v>99.2242372997781</v>
+        <v>49.2185205539928</v>
       </c>
       <c r="G22" s="6">
         <f t="shared" si="4"/>
-        <v>1101.91126685543</v>
+        <v>610.888696287793</v>
       </c>
       <c r="H22" s="6">
         <f t="shared" si="5"/>
-        <v>38.0187144461486</v>
+        <v>27.6475808094251</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B23" s="6">
         <f t="shared" si="6"/>
-        <v>1101.91126685543</v>
+        <v>610.888696287793</v>
       </c>
       <c r="C23" s="5">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="D23" s="6">
         <f t="shared" si="1"/>
-        <v>165.286690028315</v>
+        <v>85.524417480291</v>
       </c>
       <c r="E23" s="5">
         <f t="shared" si="2"/>
-        <v>0.633333333333333</v>
+        <v>0.607142857142857</v>
       </c>
       <c r="F23" s="6">
         <f t="shared" si="3"/>
-        <v>104.681570351266</v>
+        <v>51.9255391844624</v>
       </c>
       <c r="G23" s="6">
         <f t="shared" si="4"/>
-        <v>1162.51638653248</v>
+        <v>644.487574583621</v>
       </c>
       <c r="H23" s="6">
         <f t="shared" si="5"/>
-        <v>34.9729845184279</v>
+        <v>26.495026560742</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="7">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" s="6">
         <f t="shared" si="6"/>
-        <v>1162.51638653248</v>
+        <v>644.487574583621</v>
       </c>
       <c r="C24" s="5">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="D24" s="6">
         <f t="shared" si="1"/>
-        <v>174.377457979872</v>
+        <v>90.228260441707</v>
       </c>
       <c r="E24" s="5">
         <f t="shared" si="2"/>
-        <v>0.633333333333333</v>
+        <v>0.607142857142857</v>
       </c>
       <c r="F24" s="6">
         <f t="shared" si="3"/>
-        <v>110.439056720585</v>
+        <v>54.7814438396078</v>
       </c>
       <c r="G24" s="6">
         <f t="shared" si="4"/>
-        <v>1226.45478779177</v>
+        <v>679.93439118572</v>
       </c>
       <c r="H24" s="6">
         <f t="shared" si="5"/>
-        <v>32.1712520779382</v>
+        <v>25.3905192390329</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25" s="6">
         <f t="shared" si="6"/>
-        <v>1226.45478779177</v>
+        <v>679.93439118572</v>
       </c>
       <c r="C25" s="5">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="D25" s="6">
         <f t="shared" si="1"/>
-        <v>183.968218168765</v>
+        <v>95.1908147660009</v>
       </c>
       <c r="E25" s="5">
         <f t="shared" si="2"/>
-        <v>0.633333333333333</v>
+        <v>0.607142857142857</v>
       </c>
       <c r="F25" s="6">
         <f t="shared" si="3"/>
-        <v>116.513204840218</v>
+        <v>57.7944232507862</v>
       </c>
       <c r="G25" s="6">
         <f t="shared" si="4"/>
-        <v>1293.90980112031</v>
+        <v>717.330782700935</v>
       </c>
       <c r="H25" s="6">
         <f t="shared" si="5"/>
-        <v>29.5939701605074</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>39</v>
+        <v>24.3320558954611</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="7">
+        <v>10</v>
+      </c>
+      <c r="B26" s="6">
+        <f t="shared" si="6"/>
+        <v>717.330782700935</v>
+      </c>
+      <c r="C26" s="5">
+        <f t="shared" si="0"/>
+        <v>0.14</v>
+      </c>
+      <c r="D26" s="6">
+        <f t="shared" si="1"/>
+        <v>100.426309578131</v>
+      </c>
+      <c r="E26" s="5">
+        <f t="shared" si="2"/>
+        <v>0.607142857142857</v>
+      </c>
+      <c r="F26" s="6">
+        <f t="shared" si="3"/>
+        <v>60.9731165295795</v>
+      </c>
+      <c r="G26" s="6">
+        <f t="shared" si="4"/>
+        <v>756.783975749486</v>
+      </c>
+      <c r="H26" s="6">
+        <f t="shared" si="5"/>
+        <v>23.3177170788096</v>
       </c>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B28" s="6">
-        <f>SUM(H16:H25)</f>
-        <v>233.637684330237</v>
+      <c r="B28" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B29" s="19">
-        <f>(B10-B11)/(B6-B11)</f>
-        <v>1.03398074314264</v>
+        <v>104</v>
+      </c>
+      <c r="B29" s="6">
+        <f>SUM(H17:H26)</f>
+        <v>211.596764842919</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="B30" s="6">
-        <f>G25*B29</f>
-        <v>1337.87781772193</v>
+      <c r="B30" s="19">
+        <f>($B$10-$B$11)/($B$6-$B$11)</f>
+        <v>1.85212139805967</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="7" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="B31" s="6">
-        <f>B30/(1+B6)^10</f>
-        <v>339.816557877402</v>
+        <f>G26*B30</f>
+        <v>1401.6557951943</v>
       </c>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B32" s="17">
-        <f>B28+B31</f>
-        <v>573.454242207638</v>
+      <c r="B32" s="6">
+        <f>B31/(1+$B$6)^10</f>
+        <v>536.029895377893</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="B33" s="6">
-        <f>B12</f>
-        <v>1310.6</v>
+      <c r="A33" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" s="17">
+        <f>B29+B32</f>
+        <v>747.626660220812</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B34" s="5">
-        <f>B32/B33-1</f>
-        <v>-0.562449075074288</v>
+        <v>98</v>
+      </c>
+      <c r="B34" s="6">
+        <f>$B$12</f>
+        <v>1759.8</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="B35" s="19">
-        <f>B32/B5</f>
-        <v>1.08814846718717</v>
+        <v>108</v>
+      </c>
+      <c r="B35" s="5">
+        <f>B33/B34-1</f>
+        <v>-0.575163848039089</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -3421,40 +3235,611 @@
         <v>130</v>
       </c>
       <c r="B36" s="19">
-        <f>B33/B5</f>
-        <v>2.48690702087287</v>
+        <f>B33/$B$5</f>
+        <v>2.14835247189888</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="B37" s="5">
-        <f>(B6*B36-Inputs!D23)/(B36-1)</f>
-        <v>0.138725372577846</v>
+      <c r="B37" s="19">
+        <f>B34/$B$5</f>
+        <v>5.05689655172414</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="B38" s="6">
-        <f>B9*B8*B5/(B6-B8*(1-B9))*(1-((1+B8*(1-B9))/(1+B6))^B7)+B5*(1+B8*(1-B9))^B7*(B10-B11)/(B6-B11)/(1+B6)^B7</f>
-        <v>573.454242207639</v>
+      <c r="B38" s="5">
+        <f>($B$6*B37-$B$13)/(B37-1)</f>
+        <v>0.0863238876158096</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B39" s="20">
-        <f>ROUND(B32-B38,6)</f>
+        <v>133</v>
+      </c>
+      <c r="B39" s="6">
+        <f>$B$9*$B$8*$B$5/($B$6-$B$8*(1-$B$9))*(1-((1+$B$8*(1-$B$9))/(1+$B$6))^$B$7)+$B$5*(1+$B$8*(1-$B$9))^$B$7*($B$10-$B$11)/($B$6-$B$11)/(1+$B$6)^$B$7</f>
+        <v>747.626660220812</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" s="20">
+        <f>ROUND(B33-B39,6)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="9" t="s">
+    <row r="44" ht="15" spans="1:2">
+      <c r="A44" s="22" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" s="3">
+        <f>Inputs!D22</f>
+        <v>527</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" s="4">
+        <f>Inputs!D15</f>
+        <v>0.14672924</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B47" s="23">
+        <f>Inputs!D26</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B48" s="4">
+        <f>Inputs!D28</f>
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B49" s="4">
+        <f>Inputs!D29</f>
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B50" s="4">
+        <f>Inputs!D30</f>
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" s="4">
+        <f>Inputs!D31</f>
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" s="3">
+        <f>Inputs!D13</f>
+        <v>1350.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B53" s="4">
+        <f>Inputs!D23</f>
+        <v>0.159</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B54" s="5">
+        <f>1-$B$51/$B$50</f>
+        <v>0.633333333333333</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" s="7">
+        <v>1</v>
+      </c>
+      <c r="B57" s="6">
+        <f>$B$45</f>
+        <v>527</v>
+      </c>
+      <c r="C57" s="5">
+        <f t="shared" ref="C57:C66" si="7">IF(A57&lt;=$B$47,$B$48,$B$50)</f>
+        <v>0.16</v>
+      </c>
+      <c r="D57" s="6">
+        <f t="shared" ref="D57:D66" si="8">B57*C57</f>
+        <v>84.32</v>
+      </c>
+      <c r="E57" s="5">
+        <f t="shared" ref="E57:E66" si="9">IF(A57&lt;=$B$47,$B$49,$B$54)</f>
+        <v>0.16</v>
+      </c>
+      <c r="F57" s="6">
+        <f t="shared" ref="F57:F66" si="10">D57*E57</f>
+        <v>13.4912</v>
+      </c>
+      <c r="G57" s="6">
+        <f t="shared" ref="G57:G66" si="11">B57+D57-F57</f>
+        <v>597.8288</v>
+      </c>
+      <c r="H57" s="6">
+        <f t="shared" ref="H57:H66" si="12">F57/(1+$B$46)^A57</f>
+        <v>11.7649393853426</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58" s="7">
+        <v>2</v>
+      </c>
+      <c r="B58" s="6">
+        <f t="shared" ref="B58:B66" si="13">G57</f>
+        <v>597.8288</v>
+      </c>
+      <c r="C58" s="5">
+        <f t="shared" si="7"/>
+        <v>0.16</v>
+      </c>
+      <c r="D58" s="6">
+        <f t="shared" si="8"/>
+        <v>95.652608</v>
+      </c>
+      <c r="E58" s="5">
+        <f t="shared" si="9"/>
+        <v>0.16</v>
+      </c>
+      <c r="F58" s="6">
+        <f t="shared" si="10"/>
+        <v>15.30441728</v>
+      </c>
+      <c r="G58" s="6">
+        <f t="shared" si="11"/>
+        <v>678.17699072</v>
+      </c>
+      <c r="H58" s="6">
+        <f t="shared" si="12"/>
+        <v>11.6384467869091</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59" s="7">
+        <v>3</v>
+      </c>
+      <c r="B59" s="6">
+        <f t="shared" si="13"/>
+        <v>678.17699072</v>
+      </c>
+      <c r="C59" s="5">
+        <f t="shared" si="7"/>
+        <v>0.16</v>
+      </c>
+      <c r="D59" s="6">
+        <f t="shared" si="8"/>
+        <v>108.5083185152</v>
+      </c>
+      <c r="E59" s="5">
+        <f t="shared" si="9"/>
+        <v>0.16</v>
+      </c>
+      <c r="F59" s="6">
+        <f t="shared" si="10"/>
+        <v>17.361330962432</v>
+      </c>
+      <c r="G59" s="6">
+        <f t="shared" si="11"/>
+        <v>769.323978272768</v>
+      </c>
+      <c r="H59" s="6">
+        <f t="shared" si="12"/>
+        <v>11.5133141935664</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" s="7">
+        <v>4</v>
+      </c>
+      <c r="B60" s="6">
+        <f t="shared" si="13"/>
+        <v>769.323978272768</v>
+      </c>
+      <c r="C60" s="5">
+        <f t="shared" si="7"/>
+        <v>0.16</v>
+      </c>
+      <c r="D60" s="6">
+        <f t="shared" si="8"/>
+        <v>123.091836523643</v>
+      </c>
+      <c r="E60" s="5">
+        <f t="shared" si="9"/>
+        <v>0.16</v>
+      </c>
+      <c r="F60" s="6">
+        <f t="shared" si="10"/>
+        <v>19.6946938437829</v>
+      </c>
+      <c r="G60" s="6">
+        <f t="shared" si="11"/>
+        <v>872.721120952628</v>
+      </c>
+      <c r="H60" s="6">
+        <f t="shared" si="12"/>
+        <v>11.3895269830058</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" s="7">
+        <v>5</v>
+      </c>
+      <c r="B61" s="6">
+        <f t="shared" si="13"/>
+        <v>872.721120952628</v>
+      </c>
+      <c r="C61" s="5">
+        <f t="shared" si="7"/>
+        <v>0.16</v>
+      </c>
+      <c r="D61" s="6">
+        <f t="shared" si="8"/>
+        <v>139.63537935242</v>
+      </c>
+      <c r="E61" s="5">
+        <f t="shared" si="9"/>
+        <v>0.16</v>
+      </c>
+      <c r="F61" s="6">
+        <f t="shared" si="10"/>
+        <v>22.3416606963873</v>
+      </c>
+      <c r="G61" s="6">
+        <f t="shared" si="11"/>
+        <v>990.014839608661</v>
+      </c>
+      <c r="H61" s="6">
+        <f t="shared" si="12"/>
+        <v>11.2670706901324</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" s="7">
+        <v>6</v>
+      </c>
+      <c r="B62" s="6">
+        <f t="shared" si="13"/>
+        <v>990.014839608661</v>
+      </c>
+      <c r="C62" s="5">
+        <f t="shared" si="7"/>
+        <v>0.15</v>
+      </c>
+      <c r="D62" s="6">
+        <f t="shared" si="8"/>
+        <v>148.502225941299</v>
+      </c>
+      <c r="E62" s="5">
+        <f t="shared" si="9"/>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="F62" s="6">
+        <f t="shared" si="10"/>
+        <v>94.0514097628228</v>
+      </c>
+      <c r="G62" s="6">
+        <f t="shared" si="11"/>
+        <v>1044.46565578714</v>
+      </c>
+      <c r="H62" s="6">
+        <f t="shared" si="12"/>
+        <v>41.361853340259</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" s="7">
+        <v>7</v>
+      </c>
+      <c r="B63" s="6">
+        <f t="shared" si="13"/>
+        <v>1044.46565578714</v>
+      </c>
+      <c r="C63" s="5">
+        <f t="shared" si="7"/>
+        <v>0.15</v>
+      </c>
+      <c r="D63" s="6">
+        <f t="shared" si="8"/>
+        <v>156.669848368071</v>
+      </c>
+      <c r="E63" s="5">
+        <f t="shared" si="9"/>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="F63" s="6">
+        <f t="shared" si="10"/>
+        <v>99.2242372997781</v>
+      </c>
+      <c r="G63" s="6">
+        <f t="shared" si="11"/>
+        <v>1101.91126685543</v>
+      </c>
+      <c r="H63" s="6">
+        <f t="shared" si="12"/>
+        <v>38.0532332758631</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" s="7">
+        <v>8</v>
+      </c>
+      <c r="B64" s="6">
+        <f t="shared" si="13"/>
+        <v>1101.91126685543</v>
+      </c>
+      <c r="C64" s="5">
+        <f t="shared" si="7"/>
+        <v>0.15</v>
+      </c>
+      <c r="D64" s="6">
+        <f t="shared" si="8"/>
+        <v>165.286690028315</v>
+      </c>
+      <c r="E64" s="5">
+        <f t="shared" si="9"/>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="F64" s="6">
+        <f t="shared" si="10"/>
+        <v>104.681570351266</v>
+      </c>
+      <c r="G64" s="6">
+        <f t="shared" si="11"/>
+        <v>1162.51638653248</v>
+      </c>
+      <c r="H64" s="6">
+        <f t="shared" si="12"/>
+        <v>35.0092765629972</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" s="7">
+        <v>9</v>
+      </c>
+      <c r="B65" s="6">
+        <f t="shared" si="13"/>
+        <v>1162.51638653248</v>
+      </c>
+      <c r="C65" s="5">
+        <f t="shared" si="7"/>
+        <v>0.15</v>
+      </c>
+      <c r="D65" s="6">
+        <f t="shared" si="8"/>
+        <v>174.377457979872</v>
+      </c>
+      <c r="E65" s="5">
+        <f t="shared" si="9"/>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="F65" s="6">
+        <f t="shared" si="10"/>
+        <v>110.439056720585</v>
+      </c>
+      <c r="G65" s="6">
+        <f t="shared" si="11"/>
+        <v>1226.45478779177</v>
+      </c>
+      <c r="H65" s="6">
+        <f t="shared" si="12"/>
+        <v>32.2088122336203</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" s="7">
+        <v>10</v>
+      </c>
+      <c r="B66" s="6">
+        <f t="shared" si="13"/>
+        <v>1226.45478779177</v>
+      </c>
+      <c r="C66" s="5">
+        <f t="shared" si="7"/>
+        <v>0.15</v>
+      </c>
+      <c r="D66" s="6">
+        <f t="shared" si="8"/>
+        <v>183.968218168765</v>
+      </c>
+      <c r="E66" s="5">
+        <f t="shared" si="9"/>
+        <v>0.633333333333333</v>
+      </c>
+      <c r="F66" s="6">
+        <f t="shared" si="10"/>
+        <v>116.513204840218</v>
+      </c>
+      <c r="G66" s="6">
+        <f t="shared" si="11"/>
+        <v>1293.90980112031</v>
+      </c>
+      <c r="H66" s="6">
+        <f t="shared" si="12"/>
+        <v>29.6323628291447</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B69" s="6">
+        <f>SUM(H57:H66)</f>
+        <v>233.838836280841</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B70" s="19">
+        <f>($B$50-$B$51)/($B$46-$B$51)</f>
+        <v>1.03565667828492</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B71" s="6">
+        <f>G66*B70</f>
+        <v>1340.04632662856</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B72" s="6">
+        <f>B71/(1+$B$46)^10</f>
+        <v>340.808915289691</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B73" s="17">
+        <f>B69+B72</f>
+        <v>574.647751570531</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B74" s="6">
+        <f>$B$52</f>
+        <v>1350.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B75" s="5">
+        <f>B73/B74-1</f>
+        <v>-0.574492594172135</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B76" s="19">
+        <f>B73/$B$45</f>
+        <v>1.09041319083592</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B77" s="19">
+        <f>B74/$B$45</f>
+        <v>2.56261859582543</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B78" s="5">
+        <f>($B$46*B77-$B$53)/(B77-1)</f>
+        <v>0.13887654962963</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79" s="7" t="s">
         <v>133</v>
+      </c>
+      <c r="B79" s="6">
+        <f>$B$49*$B$48*$B$45/($B$46-$B$48*(1-$B$49))*(1-((1+$B$48*(1-$B$49))/(1+$B$46))^$B$47)+$B$45*(1+$B$48*(1-$B$49))^$B$47*($B$50-$B$51)/($B$46-$B$51)/(1+$B$46)^$B$47</f>
+        <v>574.647751570531</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B80" s="20">
+        <f>ROUND(B73-B79,6)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3499,7 +3884,7 @@
         <v>138</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -3550,7 +3935,7 @@
       </c>
       <c r="B10" s="3">
         <f>Inputs!B17</f>
-        <v>46.9565217391304</v>
+        <v>47.618925831202</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -3559,7 +3944,7 @@
       </c>
       <c r="B11" s="17">
         <f>B9*B10</f>
-        <v>2075.47826086957</v>
+        <v>2104.75652173913</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -3575,7 +3960,7 @@
         <v>138</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -3583,10 +3968,10 @@
         <v>146</v>
       </c>
       <c r="B15" s="14">
-        <v>14</v>
+        <v>29.9</v>
       </c>
       <c r="C15" s="15">
-        <v>2075</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -3594,10 +3979,10 @@
         <v>147</v>
       </c>
       <c r="B16" s="14">
-        <v>18.6</v>
+        <v>32.3</v>
       </c>
       <c r="C16" s="15">
-        <v>1243</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -3605,10 +3990,10 @@
         <v>148</v>
       </c>
       <c r="B17" s="14">
-        <v>11.9</v>
+        <v>82.2</v>
       </c>
       <c r="C17" s="15">
-        <v>159</v>
+        <v>9224</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -3617,7 +4002,7 @@
       </c>
       <c r="B18" s="16">
         <f>MEDIAN(B15:B17)</f>
-        <v>14</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -3626,7 +4011,7 @@
       </c>
       <c r="B19" s="3">
         <f>Inputs!C17</f>
-        <v>76.6666666666667</v>
+        <v>52.688622754491</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -3635,7 +4020,7 @@
       </c>
       <c r="B20" s="17">
         <f>B18*B19</f>
-        <v>1073.33333333333</v>
+        <v>1701.84251497006</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -3651,13 +4036,13 @@
         <v>138</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>152</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>153</v>
@@ -3811,7 +4196,7 @@
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3858,140 +4243,140 @@
     <row r="6" spans="1:6">
       <c r="A6" s="11">
         <f>Inputs!$B$15+(-0.02)</f>
-        <v>0.07770732</v>
+        <v>0.07779228</v>
       </c>
       <c r="B6" s="12">
         <f>IF(B$5&lt;$A6,Inputs!$B$20*(1+Inputs!$B$27)/($A6-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A6))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+B$5)/(($A6-B$5)*(1+$A6)^Inputs!$B$26),"")</f>
-        <v>1291.59702395244</v>
+        <v>1288.66830514103</v>
       </c>
       <c r="C6" s="12">
         <f>IF(C$5&lt;$A6,Inputs!$B$20*(1+Inputs!$B$27)/($A6-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A6))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+C$5)/(($A6-C$5)*(1+$A6)^Inputs!$B$26),"")</f>
-        <v>1464.41893061508</v>
+        <v>1460.60072205549</v>
       </c>
       <c r="D6" s="12">
         <f>IF(D$5&lt;$A6,Inputs!$B$20*(1+Inputs!$B$27)/($A6-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A6))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+D$5)/(($A6-D$5)*(1+$A6)^Inputs!$B$26),"")</f>
-        <v>1699.61493432595</v>
+        <v>1694.39651142967</v>
       </c>
       <c r="E6" s="12">
         <f>IF(E$5&lt;$A6,Inputs!$B$20*(1+Inputs!$B$27)/($A6-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A6))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+E$5)/(($A6-E$5)*(1+$A6)^Inputs!$B$26),"")</f>
-        <v>2038.3881121423</v>
+        <v>2030.76904581321</v>
       </c>
       <c r="F6" s="12">
         <f>IF(F$5&lt;$A6,Inputs!$B$20*(1+Inputs!$B$27)/($A6-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A6))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+F$5)/(($A6-F$5)*(1+$A6)^Inputs!$B$26),"")</f>
-        <v>2568.47944415497</v>
+        <v>2556.19690890309</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="11">
         <f>Inputs!$B$15+(-0.01)</f>
-        <v>0.08770732</v>
+        <v>0.08779228</v>
       </c>
       <c r="B7" s="12">
         <f>IF(B$5&lt;$A7,Inputs!$B$20*(1+Inputs!$B$27)/($A7-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A7))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+B$5)/(($A7-B$5)*(1+$A7)^Inputs!$B$26),"")</f>
-        <v>1018.56477367808</v>
+        <v>1016.73494202558</v>
       </c>
       <c r="C7" s="12">
         <f>IF(C$5&lt;$A7,Inputs!$B$20*(1+Inputs!$B$27)/($A7-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A7))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+C$5)/(($A7-C$5)*(1+$A7)^Inputs!$B$26),"")</f>
-        <v>1119.38257107891</v>
+        <v>1117.14233336539</v>
       </c>
       <c r="D7" s="12">
         <f>IF(D$5&lt;$A7,Inputs!$B$20*(1+Inputs!$B$27)/($A7-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A7))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+D$5)/(($A7-D$5)*(1+$A7)^Inputs!$B$26),"")</f>
-        <v>1246.93729844475</v>
+        <v>1244.11795275067</v>
       </c>
       <c r="E7" s="12">
         <f>IF(E$5&lt;$A7,Inputs!$B$20*(1+Inputs!$B$27)/($A7-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A7))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+E$5)/(($A7-E$5)*(1+$A7)^Inputs!$B$26),"")</f>
-        <v>1413.49085768243</v>
+        <v>1409.81476486341</v>
       </c>
       <c r="F7" s="12">
         <f>IF(F$5&lt;$A7,Inputs!$B$20*(1+Inputs!$B$27)/($A7-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A7))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+F$5)/(($A7-F$5)*(1+$A7)^Inputs!$B$26),"")</f>
-        <v>1640.15617050642</v>
+        <v>1635.13130307014</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="11">
         <f>Inputs!$B$15+(0)</f>
-        <v>0.09770732</v>
+        <v>0.09779228</v>
       </c>
       <c r="B8" s="12">
         <f>IF(B$5&lt;$A8,Inputs!$B$20*(1+Inputs!$B$27)/($A8-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A8))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+B$5)/(($A8-B$5)*(1+$A8)^Inputs!$B$26),"")</f>
-        <v>840.227423062342</v>
+        <v>838.976951827775</v>
       </c>
       <c r="C8" s="12">
         <f>IF(C$5&lt;$A8,Inputs!$B$20*(1+Inputs!$B$27)/($A8-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A8))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+C$5)/(($A8-C$5)*(1+$A8)^Inputs!$B$26),"")</f>
-        <v>905.33397093348</v>
+        <v>903.86307293379</v>
       </c>
       <c r="D8" s="12">
         <f>IF(D$5&lt;$A8,Inputs!$B$20*(1+Inputs!$B$27)/($A8-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A8))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+D$5)/(($A8-D$5)*(1+$A8)^Inputs!$B$26),"")</f>
-        <v>984.087595997622</v>
+        <v>982.325889084699</v>
       </c>
       <c r="E8" s="13">
         <f>IF(E$5&lt;$A8,Inputs!$B$20*(1+Inputs!$B$27)/($A8-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A8))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+E$5)/(($A8-E$5)*(1+$A8)^Inputs!$B$26),"")</f>
-        <v>1081.28153177762</v>
+        <v>1079.12444620358</v>
       </c>
       <c r="F8" s="12">
         <f>IF(F$5&lt;$A8,Inputs!$B$20*(1+Inputs!$B$27)/($A8-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A8))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+F$5)/(($A8-F$5)*(1+$A8)^Inputs!$B$26),"")</f>
-        <v>1204.25134762016</v>
+        <v>1201.53631829549</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="11">
         <f>Inputs!$B$15+(0.01)</f>
-        <v>0.10770732</v>
+        <v>0.10779228</v>
       </c>
       <c r="B9" s="12">
         <f>IF(B$5&lt;$A9,Inputs!$B$20*(1+Inputs!$B$27)/($A9-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A9))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+B$5)/(($A9-B$5)*(1+$A9)^Inputs!$B$26),"")</f>
-        <v>714.62449512987</v>
+        <v>713.716350740097</v>
       </c>
       <c r="C9" s="12">
         <f>IF(C$5&lt;$A9,Inputs!$B$20*(1+Inputs!$B$27)/($A9-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A9))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+C$5)/(($A9-C$5)*(1+$A9)^Inputs!$B$26),"")</f>
-        <v>759.604425921308</v>
+        <v>758.565366766303</v>
       </c>
       <c r="D9" s="12">
         <f>IF(D$5&lt;$A9,Inputs!$B$20*(1+Inputs!$B$27)/($A9-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A9))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+D$5)/(($A9-D$5)*(1+$A9)^Inputs!$B$26),"")</f>
-        <v>812.378849818897</v>
+        <v>811.17476463351</v>
       </c>
       <c r="E9" s="12">
         <f>IF(E$5&lt;$A9,Inputs!$B$20*(1+Inputs!$B$27)/($A9-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A9))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+E$5)/(($A9-E$5)*(1+$A9)^Inputs!$B$26),"")</f>
-        <v>875.166005135497</v>
+        <v>873.749520668087</v>
       </c>
       <c r="F9" s="12">
         <f>IF(F$5&lt;$A9,Inputs!$B$20*(1+Inputs!$B$27)/($A9-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A9))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+F$5)/(($A9-F$5)*(1+$A9)^Inputs!$B$26),"")</f>
-        <v>951.114066433946</v>
+        <v>949.41734446059</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="11">
         <f>Inputs!$B$15+(0.02)</f>
-        <v>0.11770732</v>
+        <v>0.11779228</v>
       </c>
       <c r="B10" s="12">
         <f>IF(B$5&lt;$A10,Inputs!$B$20*(1+Inputs!$B$27)/($A10-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A10))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+B$5)/(($A10-B$5)*(1+$A10)^Inputs!$B$26),"")</f>
-        <v>621.394887343001</v>
+        <v>620.705684674414</v>
       </c>
       <c r="C10" s="12">
         <f>IF(C$5&lt;$A10,Inputs!$B$20*(1+Inputs!$B$27)/($A10-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A10))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+C$5)/(($A10-C$5)*(1+$A10)^Inputs!$B$26),"")</f>
-        <v>654.002597413008</v>
+        <v>653.229875702292</v>
       </c>
       <c r="D10" s="12">
         <f>IF(D$5&lt;$A10,Inputs!$B$20*(1+Inputs!$B$27)/($A10-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A10))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+D$5)/(($A10-D$5)*(1+$A10)^Inputs!$B$26),"")</f>
-        <v>691.426287508515</v>
+        <v>690.551691331065</v>
       </c>
       <c r="E10" s="12">
         <f>IF(E$5&lt;$A10,Inputs!$B$20*(1+Inputs!$B$27)/($A10-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A10))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+E$5)/(($A10-E$5)*(1+$A10)^Inputs!$B$26),"")</f>
-        <v>734.817971467498</v>
+        <v>733.817201889975</v>
       </c>
       <c r="F10" s="12">
         <f>IF(F$5&lt;$A10,Inputs!$B$20*(1+Inputs!$B$27)/($A10-Inputs!$B$27)*(1-((1+Inputs!$B$27)/(1+$A10))^Inputs!$B$26)+Inputs!$B$20*(1+Inputs!$B$27)^Inputs!$B$26*(1+F$5)/(($A10-F$5)*(1+$A10)^Inputs!$B$26),"")</f>
-        <v>785.72892403209</v>
+        <v>784.569094809801</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B11" s="3">
         <f>Inputs!B13</f>
-        <v>1836</v>
+        <v>1861.9</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -4027,140 +4412,140 @@
     <row r="16" spans="1:6">
       <c r="A16" s="11">
         <f>Inputs!$C$15+(-0.02)</f>
-        <v>0.09333288</v>
+        <v>0.08089332</v>
       </c>
       <c r="B16" s="12">
-        <f>IF(B$15&lt;$A16,Inputs!$C$20*(1+Inputs!$C$27)/($A16-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A16))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+B$15)/(($A16-B$15)*(1+$A16)^Inputs!$C$26),"")</f>
-        <v>1111.67256309421</v>
+        <f>IF(B$15&lt;$A16,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A16-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A16))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-B$15)/($A16-B$15)/(1+$A16)^Inputs!$C$26,"")</f>
+        <v>1048.95234578514</v>
       </c>
       <c r="C16" s="12">
-        <f>IF(C$15&lt;$A16,Inputs!$C$20*(1+Inputs!$C$27)/($A16-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A16))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+C$15)/(($A16-C$15)*(1+$A16)^Inputs!$C$26),"")</f>
-        <v>1207.41019324622</v>
+        <f>IF(C$15&lt;$A16,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A16-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A16))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-C$15)/($A16-C$15)/(1+$A16)^Inputs!$C$26,"")</f>
+        <v>1127.97216532017</v>
       </c>
       <c r="D16" s="12">
-        <f>IF(D$15&lt;$A16,Inputs!$C$20*(1+Inputs!$C$27)/($A16-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A16))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+D$15)/(($A16-D$15)*(1+$A16)^Inputs!$C$26),"")</f>
-        <v>1325.2413537964</v>
+        <f>IF(D$15&lt;$A16,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A16-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A16))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-D$15)/($A16-D$15)/(1+$A16)^Inputs!$C$26,"")</f>
+        <v>1232.57027153174</v>
       </c>
       <c r="E16" s="12">
-        <f>IF(E$15&lt;$A16,Inputs!$C$20*(1+Inputs!$C$27)/($A16-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A16))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+E$15)/(($A16-E$15)*(1+$A16)^Inputs!$C$26),"")</f>
-        <v>1473.81144148959</v>
+        <f>IF(E$15&lt;$A16,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A16-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A16))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-E$15)/($A16-E$15)/(1+$A16)^Inputs!$C$26,"")</f>
+        <v>1377.56416561894</v>
       </c>
       <c r="F16" s="12">
-        <f>IF(F$15&lt;$A16,Inputs!$C$20*(1+Inputs!$C$27)/($A16-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A16))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+F$15)/(($A16-F$15)*(1+$A16)^Inputs!$C$26),"")</f>
-        <v>1666.95316166494</v>
+        <f>IF(F$15&lt;$A16,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A16-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A16))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-F$15)/($A16-F$15)/(1+$A16)^Inputs!$C$26,"")</f>
+        <v>1591.95530920369</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="11">
         <f>Inputs!$C$15+(-0.01)</f>
-        <v>0.10333288</v>
+        <v>0.09089332</v>
       </c>
       <c r="B17" s="12">
-        <f>IF(B$15&lt;$A17,Inputs!$C$20*(1+Inputs!$C$27)/($A17-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A17))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+B$15)/(($A17-B$15)*(1+$A17)^Inputs!$C$26),"")</f>
-        <v>933.519234979394</v>
+        <f>IF(B$15&lt;$A17,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A17-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A17))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-B$15)/($A17-B$15)/(1+$A17)^Inputs!$C$26,"")</f>
+        <v>823.21300502212</v>
       </c>
       <c r="C17" s="12">
-        <f>IF(C$15&lt;$A17,Inputs!$C$20*(1+Inputs!$C$27)/($A17-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A17))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+C$15)/(($A17-C$15)*(1+$A17)^Inputs!$C$26),"")</f>
-        <v>997.930394930124</v>
+        <f>IF(C$15&lt;$A17,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A17-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A17))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-C$15)/($A17-C$15)/(1+$A17)^Inputs!$C$26,"")</f>
+        <v>862.613214974082</v>
       </c>
       <c r="D17" s="12">
-        <f>IF(D$15&lt;$A17,Inputs!$C$20*(1+Inputs!$C$27)/($A17-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A17))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+D$15)/(($A17-D$15)*(1+$A17)^Inputs!$C$26),"")</f>
-        <v>1074.41875002778</v>
+        <f>IF(D$15&lt;$A17,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A17-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A17))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-D$15)/($A17-D$15)/(1+$A17)^Inputs!$C$26,"")</f>
+        <v>911.648301710801</v>
       </c>
       <c r="E17" s="12">
-        <f>IF(E$15&lt;$A17,Inputs!$C$20*(1+Inputs!$C$27)/($A17-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A17))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+E$15)/(($A17-E$15)*(1+$A17)^Inputs!$C$26),"")</f>
-        <v>1166.73243047282</v>
+        <f>IF(E$15&lt;$A17,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A17-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A17))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-E$15)/($A17-E$15)/(1+$A17)^Inputs!$C$26,"")</f>
+        <v>974.344728980164</v>
       </c>
       <c r="F17" s="12">
-        <f>IF(F$15&lt;$A17,Inputs!$C$20*(1+Inputs!$C$27)/($A17-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A17))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+F$15)/(($A17-F$15)*(1+$A17)^Inputs!$C$26),"")</f>
-        <v>1280.34949080977</v>
+        <f>IF(F$15&lt;$A17,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A17-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A17))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-F$15)/($A17-F$15)/(1+$A17)^Inputs!$C$26,"")</f>
+        <v>1057.33564945044</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="11">
         <f>Inputs!$C$15+(0)</f>
-        <v>0.11333288</v>
+        <v>0.10089332</v>
       </c>
       <c r="B18" s="12">
-        <f>IF(B$15&lt;$A18,Inputs!$C$20*(1+Inputs!$C$27)/($A18-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A18))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+B$15)/(($A18-B$15)*(1+$A18)^Inputs!$C$26),"")</f>
-        <v>804.033767923981</v>
+        <f>IF(B$15&lt;$A18,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A18-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A18))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-B$15)/($A18-B$15)/(1+$A18)^Inputs!$C$26,"")</f>
+        <v>672.463241703294</v>
       </c>
       <c r="C18" s="12">
-        <f>IF(C$15&lt;$A18,Inputs!$C$20*(1+Inputs!$C$27)/($A18-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A18))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+C$15)/(($A18-C$15)*(1+$A18)^Inputs!$C$26),"")</f>
-        <v>849.83755758176</v>
+        <f>IF(C$15&lt;$A18,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A18-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A18))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-C$15)/($A18-C$15)/(1+$A18)^Inputs!$C$26,"")</f>
+        <v>693.035162273399</v>
       </c>
       <c r="D18" s="12">
-        <f>IF(D$15&lt;$A18,Inputs!$C$20*(1+Inputs!$C$27)/($A18-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A18))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+D$15)/(($A18-D$15)*(1+$A18)^Inputs!$C$26),"")</f>
-        <v>902.87357632146</v>
+        <f>IF(D$15&lt;$A18,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A18-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A18))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-D$15)/($A18-D$15)/(1+$A18)^Inputs!$C$26,"")</f>
+        <v>717.649248017658</v>
       </c>
       <c r="E18" s="13">
-        <f>IF(E$15&lt;$A18,Inputs!$C$20*(1+Inputs!$C$27)/($A18-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A18))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+E$15)/(($A18-E$15)*(1+$A18)^Inputs!$C$26),"")</f>
-        <v>965.00155464548</v>
+        <f>IF(E$15&lt;$A18,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A18-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A18))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-E$15)/($A18-E$15)/(1+$A18)^Inputs!$C$26,"")</f>
+        <v>747.626660220812</v>
       </c>
       <c r="F18" s="12">
-        <f>IF(F$15&lt;$A18,Inputs!$C$20*(1+Inputs!$C$27)/($A18-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A18))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+F$15)/(($A18-F$15)*(1+$A18)^Inputs!$C$26),"")</f>
-        <v>1038.77862792256</v>
+        <f>IF(F$15&lt;$A18,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A18-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A18))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-F$15)/($A18-F$15)/(1+$A18)^Inputs!$C$26,"")</f>
+        <v>784.934710338216</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="11">
         <f>Inputs!$C$15+(0.01)</f>
-        <v>0.12333288</v>
+        <v>0.11089332</v>
       </c>
       <c r="B19" s="12">
-        <f>IF(B$15&lt;$A19,Inputs!$C$20*(1+Inputs!$C$27)/($A19-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A19))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+B$15)/(($A19-B$15)*(1+$A19)^Inputs!$C$26),"")</f>
-        <v>705.692380063066</v>
+        <f>IF(B$15&lt;$A19,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A19-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A19))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-B$15)/($A19-B$15)/(1+$A19)^Inputs!$C$26,"")</f>
+        <v>564.925449321316</v>
       </c>
       <c r="C19" s="12">
-        <f>IF(C$15&lt;$A19,Inputs!$C$20*(1+Inputs!$C$27)/($A19-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A19))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+C$15)/(($A19-C$15)*(1+$A19)^Inputs!$C$26),"")</f>
-        <v>739.618613813524</v>
+        <f>IF(C$15&lt;$A19,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A19-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A19))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-C$15)/($A19-C$15)/(1+$A19)^Inputs!$C$26,"")</f>
+        <v>575.58806666399</v>
       </c>
       <c r="D19" s="12">
-        <f>IF(D$15&lt;$A19,Inputs!$C$20*(1+Inputs!$C$27)/($A19-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A19))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+D$15)/(($A19-D$15)*(1+$A19)^Inputs!$C$26),"")</f>
-        <v>778.171180765469</v>
+        <f>IF(D$15&lt;$A19,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A19-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A19))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-D$15)/($A19-D$15)/(1+$A19)^Inputs!$C$26,"")</f>
+        <v>588.001716360076</v>
       </c>
       <c r="E19" s="12">
-        <f>IF(E$15&lt;$A19,Inputs!$C$20*(1+Inputs!$C$27)/($A19-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A19))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+E$15)/(($A19-E$15)*(1+$A19)^Inputs!$C$26),"")</f>
-        <v>822.365624212585</v>
+        <f>IF(E$15&lt;$A19,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A19-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A19))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-E$15)/($A19-E$15)/(1+$A19)^Inputs!$C$26,"")</f>
+        <v>602.636320133697</v>
       </c>
       <c r="F19" s="12">
-        <f>IF(F$15&lt;$A19,Inputs!$C$20*(1+Inputs!$C$27)/($A19-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A19))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+F$15)/(($A19-F$15)*(1+$A19)^Inputs!$C$26),"")</f>
-        <v>873.538187626316</v>
+        <f>IF(F$15&lt;$A19,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A19-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A19))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-F$15)/($A19-F$15)/(1+$A19)^Inputs!$C$26,"")</f>
+        <v>620.14646902279</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="11">
         <f>Inputs!$C$15+(0.02)</f>
-        <v>0.13333288</v>
+        <v>0.12089332</v>
       </c>
       <c r="B20" s="12">
-        <f>IF(B$15&lt;$A20,Inputs!$C$20*(1+Inputs!$C$27)/($A20-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A20))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+B$15)/(($A20-B$15)*(1+$A20)^Inputs!$C$26),"")</f>
-        <v>628.481680211259</v>
+        <f>IF(B$15&lt;$A20,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A20-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A20))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-B$15)/($A20-B$15)/(1+$A20)^Inputs!$C$26,"")</f>
+        <v>484.538045509209</v>
       </c>
       <c r="C20" s="12">
-        <f>IF(C$15&lt;$A20,Inputs!$C$20*(1+Inputs!$C$27)/($A20-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A20))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+C$15)/(($A20-C$15)*(1+$A20)^Inputs!$C$26),"")</f>
-        <v>654.408127372122</v>
+        <f>IF(C$15&lt;$A20,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A20-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A20))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-C$15)/($A20-C$15)/(1+$A20)^Inputs!$C$26,"")</f>
+        <v>489.630501064124</v>
       </c>
       <c r="D20" s="12">
-        <f>IF(D$15&lt;$A20,Inputs!$C$20*(1+Inputs!$C$27)/($A20-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A20))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+D$15)/(($A20-D$15)*(1+$A20)^Inputs!$C$26),"")</f>
-        <v>683.445765117165</v>
+        <f>IF(D$15&lt;$A20,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A20-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A20))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-D$15)/($A20-D$15)/(1+$A20)^Inputs!$C$26,"")</f>
+        <v>495.441283191262</v>
       </c>
       <c r="E20" s="12">
-        <f>IF(E$15&lt;$A20,Inputs!$C$20*(1+Inputs!$C$27)/($A20-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A20))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+E$15)/(($A20-E$15)*(1+$A20)^Inputs!$C$26),"")</f>
-        <v>716.190356793308</v>
+        <f>IF(E$15&lt;$A20,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A20-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A20))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-E$15)/($A20-E$15)/(1+$A20)^Inputs!$C$26,"")</f>
+        <v>502.133912238109</v>
       </c>
       <c r="F20" s="12">
-        <f>IF(F$15&lt;$A20,Inputs!$C$20*(1+Inputs!$C$27)/($A20-Inputs!$C$27)*(1-((1+Inputs!$C$27)/(1+$A20))^Inputs!$C$26)+Inputs!$C$20*(1+Inputs!$C$27)^Inputs!$C$26*(1+F$15)/(($A20-F$15)*(1+$A20)^Inputs!$C$26),"")</f>
-        <v>753.400147664703</v>
+        <f>IF(F$15&lt;$A20,Inputs!$C$29*Inputs!$C$28*Inputs!$C$22/($A20-Inputs!$C$28*(1-Inputs!$C$29))*(1-((1+Inputs!$C$28*(1-Inputs!$C$29))/(1+$A20))^Inputs!$C$26)+Inputs!$C$22*(1+Inputs!$C$28*(1-Inputs!$C$29))^Inputs!$C$26*(Inputs!$C$30-F$15)/($A20-F$15)/(1+$A20)^Inputs!$C$26,"")</f>
+        <v>509.925615706724</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B21" s="3">
         <f>Inputs!C13</f>
-        <v>1035</v>
+        <v>1759.8</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -4196,140 +4581,140 @@
     <row r="26" spans="1:6">
       <c r="A26" s="11">
         <f>Inputs!$D$15+(-0.02)</f>
-        <v>0.12687792</v>
+        <v>0.12672924</v>
       </c>
       <c r="B26" s="12">
         <f>IF(B$25&lt;$A26,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A26-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A26))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-B$25)/($A26-B$25)/(1+$A26)^Inputs!$D$26,"")</f>
-        <v>750.49317689064</v>
+        <v>752.155914662847</v>
       </c>
       <c r="C26" s="12">
         <f>IF(C$25&lt;$A26,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A26-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A26))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-C$25)/($A26-C$25)/(1+$A26)^Inputs!$D$26,"")</f>
-        <v>759.347962385801</v>
+        <v>761.105057709068</v>
       </c>
       <c r="D26" s="12">
         <f>IF(D$25&lt;$A26,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A26-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A26))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-D$25)/($A26-D$25)/(1+$A26)^Inputs!$D$26,"")</f>
-        <v>769.354546146988</v>
+        <v>771.220528356895</v>
       </c>
       <c r="E26" s="12">
         <f>IF(E$25&lt;$A26,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A26-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A26))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-E$25)/($A26-E$25)/(1+$A26)^Inputs!$D$26,"")</f>
-        <v>780.75329369939</v>
+        <v>782.746228730818</v>
       </c>
       <c r="F26" s="12">
         <f>IF(F$25&lt;$A26,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A26-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A26))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-F$25)/($A26-F$25)/(1+$A26)^Inputs!$D$26,"")</f>
-        <v>793.856452446458</v>
+        <v>795.999162979114</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="11">
         <f>Inputs!$D$15+(-0.01)</f>
-        <v>0.13687792</v>
+        <v>0.13672924</v>
       </c>
       <c r="B27" s="12">
         <f>IF(B$25&lt;$A27,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A27-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A27))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-B$25)/($A27-B$25)/(1+$A27)^Inputs!$D$26,"")</f>
-        <v>650.965553548672</v>
+        <v>652.286263339797</v>
       </c>
       <c r="C27" s="12">
         <f>IF(C$25&lt;$A27,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A27-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A27))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-C$25)/($A27-C$25)/(1+$A27)^Inputs!$D$26,"")</f>
-        <v>654.808012794979</v>
+        <v>656.187091109782</v>
       </c>
       <c r="D27" s="12">
         <f>IF(D$25&lt;$A27,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A27-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A27))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-D$25)/($A27-D$25)/(1+$A27)^Inputs!$D$26,"")</f>
-        <v>659.0927546427</v>
+        <v>660.537689657187</v>
       </c>
       <c r="E27" s="12">
         <f>IF(E$25&lt;$A27,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A27-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A27))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-E$25)/($A27-E$25)/(1+$A27)^Inputs!$D$26,"")</f>
-        <v>663.900805075657</v>
+        <v>665.420606692738</v>
       </c>
       <c r="F27" s="12">
         <f>IF(F$25&lt;$A27,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A27-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A27))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-F$25)/($A27-F$25)/(1+$A27)^Inputs!$D$26,"")</f>
-        <v>669.334269207756</v>
+        <v>670.939906551258</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="11">
         <f>Inputs!$D$15+(0)</f>
-        <v>0.14687792</v>
+        <v>0.14672924</v>
       </c>
       <c r="B28" s="12">
         <f>IF(B$25&lt;$A28,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A28-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A28))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-B$25)/($A28-B$25)/(1+$A28)^Inputs!$D$26,"")</f>
-        <v>571.074708373257</v>
+        <v>572.145759111611</v>
       </c>
       <c r="C28" s="12">
         <f>IF(C$25&lt;$A28,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A28-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A28))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-C$25)/($A28-C$25)/(1+$A28)^Inputs!$D$26,"")</f>
-        <v>571.790030591826</v>
+        <v>572.897774516237</v>
       </c>
       <c r="D28" s="12">
         <f>IF(D$25&lt;$A28,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A28-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A28))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-D$25)/($A28-D$25)/(1+$A28)^Inputs!$D$26,"")</f>
-        <v>572.579190297674</v>
+        <v>573.727534293156</v>
       </c>
       <c r="E28" s="13">
         <f>IF(E$25&lt;$A28,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A28-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A28))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-E$25)/($A28-E$25)/(1+$A28)^Inputs!$D$26,"")</f>
-        <v>573.454242207639</v>
+        <v>574.647751570531</v>
       </c>
       <c r="F28" s="12">
         <f>IF(F$25&lt;$A28,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A28-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A28))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-F$25)/($A28-F$25)/(1+$A28)^Inputs!$D$26,"")</f>
-        <v>574.430016131893</v>
+        <v>575.674071158659</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="11">
         <f>Inputs!$D$15+(0.01)</f>
-        <v>0.15687792</v>
+        <v>0.15672924</v>
       </c>
       <c r="B29" s="12">
         <f>IF(B$25&lt;$A29,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A29-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A29))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-B$25)/($A29-B$25)/(1+$A29)^Inputs!$D$26,"")</f>
-        <v>505.725696131593</v>
+        <v>506.609171222441</v>
       </c>
       <c r="C29" s="12">
         <f>IF(C$25&lt;$A29,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A29-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A29))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-C$25)/($A29-C$25)/(1+$A29)^Inputs!$D$26,"")</f>
-        <v>504.469219806817</v>
+        <v>505.375860081885</v>
       </c>
       <c r="D29" s="12">
         <f>IF(D$25&lt;$A29,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A29-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A29))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-D$25)/($A29-D$25)/(1+$A29)^Inputs!$D$26,"")</f>
-        <v>503.095181657787</v>
+        <v>504.026993809432</v>
       </c>
       <c r="E29" s="12">
         <f>IF(E$25&lt;$A29,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A29-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A29))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-E$25)/($A29-E$25)/(1+$A29)^Inputs!$D$26,"")</f>
-        <v>501.586272464174</v>
+        <v>502.545533774119</v>
       </c>
       <c r="F29" s="12">
         <f>IF(F$25&lt;$A29,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A29-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A29))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-F$25)/($A29-F$25)/(1+$A29)^Inputs!$D$26,"")</f>
-        <v>499.921609596906</v>
+        <v>500.910918391435</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="11">
         <f>Inputs!$D$15+(0.02)</f>
-        <v>0.16687792</v>
+        <v>0.16672924</v>
       </c>
       <c r="B30" s="12">
         <f>IF(B$25&lt;$A30,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A30-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A30))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-B$25)/($A30-B$25)/(1+$A30)^Inputs!$D$26,"")</f>
-        <v>451.433197052034</v>
+        <v>452.172345865459</v>
       </c>
       <c r="C30" s="12">
         <f>IF(C$25&lt;$A30,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A30-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A30))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-C$25)/($A30-C$25)/(1+$A30)^Inputs!$D$26,"")</f>
-        <v>448.935772147433</v>
+        <v>449.689408472287</v>
       </c>
       <c r="D30" s="12">
         <f>IF(D$25&lt;$A30,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A30-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A30))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-D$25)/($A30-D$25)/(1+$A30)^Inputs!$D$26,"")</f>
-        <v>446.224669167059</v>
+        <v>446.993761959004</v>
       </c>
       <c r="E30" s="12">
         <f>IF(E$25&lt;$A30,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A30-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A30))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-E$25)/($A30-E$25)/(1+$A30)^Inputs!$D$26,"")</f>
-        <v>443.271239284256</v>
+        <v>444.056849460801</v>
       </c>
       <c r="F30" s="12">
         <f>IF(F$25&lt;$A30,Inputs!$D$29*Inputs!$D$28*Inputs!$D$22/($A30-Inputs!$D$28*(1-Inputs!$D$29))*(1-((1+Inputs!$D$28*(1-Inputs!$D$29))/(1+$A30))^Inputs!$D$26)+Inputs!$D$22*(1+Inputs!$D$28*(1-Inputs!$D$29))^Inputs!$D$26*(Inputs!$D$30-F$25)/($A30-F$25)/(1+$A30)^Inputs!$D$26,"")</f>
-        <v>440.041472634906</v>
+        <v>440.844762839912</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B31" s="3">
         <f>Inputs!D13</f>
-        <v>1310.6</v>
+        <v>1350.5</v>
       </c>
     </row>
   </sheetData>
@@ -4346,7 +4731,7 @@
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="6" width="14" customWidth="1"/>
     <col min="7" max="10" width="13" customWidth="1"/>
@@ -4411,23 +4796,23 @@
       </c>
       <c r="D2" s="3">
         <f>Inputs!B13</f>
-        <v>1836</v>
+        <v>1861.9</v>
       </c>
       <c r="E2" s="4">
         <f>Inputs!B15</f>
-        <v>0.09770732</v>
+        <v>0.09779228</v>
       </c>
       <c r="F2" s="3">
         <f>DDM!B29</f>
-        <v>1081.28153177762</v>
+        <v>1079.12444620358</v>
       </c>
       <c r="G2" s="5">
         <f>F2/D2-1</f>
-        <v>-0.411066703824826</v>
+        <v>-0.420417613081485</v>
       </c>
       <c r="H2" s="3">
         <f>Comps!B11</f>
-        <v>2075.47826086957</v>
+        <v>2104.75652173913</v>
       </c>
       <c r="I2" s="5">
         <f>H2/D2-1</f>
@@ -4435,15 +4820,15 @@
       </c>
       <c r="J2" s="6">
         <f>AVERAGE(F2,H2)</f>
-        <v>1578.37989632359</v>
+        <v>1591.94048397136</v>
       </c>
       <c r="K2" s="5">
         <f>J2/D2-1</f>
-        <v>-0.140315960608065</v>
+        <v>-0.144991415236395</v>
       </c>
       <c r="L2" s="4">
         <f>DDM!B33</f>
-        <v>0.0737296960681939</v>
+        <v>0.074139180268012</v>
       </c>
       <c r="M2" s="7" t="str">
         <f>IF(K2&gt;Inputs!$B$7,"Undervalued",IF(K2&lt;-Inputs!$B$7,"Overvalued","Fairly valued"))</f>
@@ -4453,55 +4838,55 @@
     <row r="3" spans="1:13">
       <c r="A3" s="2" t="str">
         <f>Inputs!C11</f>
-        <v>INFY.NS</v>
+        <v>SUNPHARMA.NS</v>
       </c>
       <c r="B3" s="2" t="str">
         <f>Inputs!C10</f>
-        <v>Infosys</v>
+        <v>Sun Pharma</v>
       </c>
       <c r="C3" s="2" t="str">
         <f>Inputs!C12</f>
-        <v>Two-stage DDM</v>
+        <v>Two-stage residual income</v>
       </c>
       <c r="D3" s="3">
         <f>Inputs!C13</f>
-        <v>1035</v>
+        <v>1759.8</v>
       </c>
       <c r="E3" s="4">
         <f>Inputs!C15</f>
-        <v>0.11333288</v>
+        <v>0.10089332</v>
       </c>
       <c r="F3" s="3">
-        <f>DDM!C29</f>
-        <v>965.00155464548</v>
+        <f>ResidualIncome!B33</f>
+        <v>747.626660220812</v>
       </c>
       <c r="G3" s="5">
         <f>F3/D3-1</f>
-        <v>-0.0676313481686179</v>
+        <v>-0.575163848039089</v>
       </c>
       <c r="H3" s="3">
         <f>Comps!B20</f>
-        <v>1073.33333333333</v>
+        <v>1701.84251497006</v>
       </c>
       <c r="I3" s="5">
         <f>H3/D3-1</f>
-        <v>0.0370370370370372</v>
+        <v>-0.0329341317365269</v>
       </c>
       <c r="J3" s="6">
         <f>AVERAGE(F3,H3)</f>
-        <v>1019.16744398941</v>
+        <v>1224.73458759544</v>
       </c>
       <c r="K3" s="5">
         <f>J3/D3-1</f>
-        <v>-0.0152971555657904</v>
+        <v>-0.304048989887808</v>
       </c>
       <c r="L3" s="4">
-        <f>DDM!C33</f>
-        <v>0.0639884864265928</v>
+        <f>ResidualIncome!B38</f>
+        <v>0.0863238876158096</v>
       </c>
       <c r="M3" s="7" t="str">
         <f>IF(K3&gt;Inputs!$B$7,"Undervalued",IF(K3&lt;-Inputs!$B$7,"Overvalued","Fairly valued"))</f>
-        <v>Fairly valued</v>
+        <v>Overvalued</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4515,23 +4900,23 @@
       </c>
       <c r="C4" s="2" t="str">
         <f>Inputs!D12</f>
-        <v>Two-stage P/B (residual income)</v>
+        <v>Two-stage residual income (bank)</v>
       </c>
       <c r="D4" s="3">
         <f>Inputs!D13</f>
-        <v>1310.6</v>
+        <v>1350.5</v>
       </c>
       <c r="E4" s="4">
         <f>Inputs!D15</f>
-        <v>0.14687792</v>
+        <v>0.14672924</v>
       </c>
       <c r="F4" s="3">
-        <f>Bank!B32</f>
-        <v>573.454242207638</v>
+        <f>ResidualIncome!B73</f>
+        <v>574.647751570531</v>
       </c>
       <c r="G4" s="5">
         <f>F4/D4-1</f>
-        <v>-0.562449075074288</v>
+        <v>-0.574492594172135</v>
       </c>
       <c r="H4" s="3">
         <f>Comps!B31</f>
@@ -4539,19 +4924,19 @@
       </c>
       <c r="I4" s="5">
         <f>H4/D4-1</f>
-        <v>-0.130900849874984</v>
+        <v>-0.156578048016404</v>
       </c>
       <c r="J4" s="6">
         <f>AVERAGE(F4,H4)</f>
-        <v>856.247794180742</v>
+        <v>856.844548862189</v>
       </c>
       <c r="K4" s="5">
         <f>J4/D4-1</f>
-        <v>-0.346674962474636</v>
+        <v>-0.36553532109427</v>
       </c>
       <c r="L4" s="4">
-        <f>Bank!B37</f>
-        <v>0.138725372577846</v>
+        <f>ResidualIncome!B78</f>
+        <v>0.13887654962963</v>
       </c>
       <c r="M4" s="7" t="str">
         <f>IF(K4&gt;Inputs!$B$7,"Undervalued",IF(K4&lt;-Inputs!$B$7,"Overvalued","Fairly valued"))</f>

</xml_diff>